<commit_message>
learning pysystemtrade. added downloading data via IB
</commit_message>
<xml_diff>
--- a/perplexity_examples/comprehensive_diagnostic_analysis.xlsx
+++ b/perplexity_examples/comprehensive_diagnostic_analysis.xlsx
@@ -564,31 +564,31 @@
         <v>20</v>
       </c>
       <c r="B2" s="6">
-        <v>43321</v>
+        <v>44111</v>
       </c>
       <c r="C2" s="6">
-        <v>45933</v>
+        <v>45936</v>
       </c>
       <c r="D2" s="2">
-        <v>1867</v>
+        <v>1304</v>
       </c>
       <c r="E2" s="2">
-        <v>1866</v>
+        <v>1303</v>
       </c>
       <c r="F2" s="2">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="G2" s="2">
-        <v>0.9630423138725228</v>
+        <v>0.9624233128834356</v>
       </c>
       <c r="J2" s="4">
-        <v>0.006580835163442976</v>
+        <v>0.006406045445478905</v>
       </c>
       <c r="K2" s="4">
-        <v>0.006976300627326518</v>
+        <v>0.006875927329392475</v>
       </c>
       <c r="L2" s="4">
-        <v>0.3985560622906569</v>
+        <v>0.3924779319617224</v>
       </c>
       <c r="M2" s="4" t="s">
         <v>23</v>
@@ -600,16 +600,16 @@
         <v>1</v>
       </c>
       <c r="Q2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R2">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="S2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T2">
-        <v>0.5380381953392962</v>
+        <v>0.3024201223873572</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -617,31 +617,31 @@
         <v>21</v>
       </c>
       <c r="B3" s="6">
-        <v>43102</v>
+        <v>44112</v>
       </c>
       <c r="C3" s="6">
-        <v>45933</v>
+        <v>45936</v>
       </c>
       <c r="D3" s="2">
-        <v>2024</v>
+        <v>1303</v>
       </c>
       <c r="E3" s="2">
-        <v>2023</v>
+        <v>1302</v>
       </c>
       <c r="F3" s="2">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="G3" s="2">
-        <v>0.9634387351778656</v>
+        <v>0.9623944742900997</v>
       </c>
       <c r="J3" s="4">
-        <v>0.004647210948420895</v>
+        <v>0.004518505279176866</v>
       </c>
       <c r="K3" s="4">
-        <v>0.005603449398603249</v>
+        <v>0.005637687130383457</v>
       </c>
       <c r="L3" s="4">
-        <v>3.343353967687355</v>
+        <v>3.363782251811863</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>23</v>
@@ -653,16 +653,16 @@
         <v>1</v>
       </c>
       <c r="Q3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R3">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="S3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T3">
-        <v>0.6297354452813277</v>
+        <v>0.4362724803457434</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -670,31 +670,31 @@
         <v>22</v>
       </c>
       <c r="B4" s="6">
-        <v>43102</v>
+        <v>44112</v>
       </c>
       <c r="C4" s="6">
-        <v>45933</v>
+        <v>45936</v>
       </c>
       <c r="D4" s="2">
-        <v>2024</v>
+        <v>1303</v>
       </c>
       <c r="E4" s="2">
-        <v>2023</v>
+        <v>1302</v>
       </c>
       <c r="F4" s="2">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="G4" s="2">
-        <v>0.9634387351778656</v>
+        <v>0.9623944742900997</v>
       </c>
       <c r="J4" s="4">
-        <v>0.002385696932113174</v>
+        <v>0.002409572359965174</v>
       </c>
       <c r="K4" s="4">
-        <v>0.002918384780843121</v>
+        <v>0.002755045394670109</v>
       </c>
       <c r="L4" s="4">
-        <v>0.1457733220296648</v>
+        <v>0.1376145195657048</v>
       </c>
       <c r="M4" s="4" t="s">
         <v>23</v>
@@ -706,16 +706,16 @@
         <v>1</v>
       </c>
       <c r="Q4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R4">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="S4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T4">
-        <v>1.819272786519806</v>
+        <v>0.5506409737245463</v>
       </c>
     </row>
   </sheetData>
@@ -750,19 +750,19 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2">
-        <v>18817.92979611094</v>
+        <v>19109.35466489224</v>
       </c>
       <c r="B2" t="s">
         <v>30</v>
       </c>
       <c r="C2">
-        <v>1.148682389459768</v>
+        <v>1.180024326165145</v>
       </c>
       <c r="D2">
-        <v>16382.18707693527</v>
+        <v>16194.03451367313</v>
       </c>
       <c r="E2">
-        <v>0.1044675195694753</v>
+        <v>0.101692818816691</v>
       </c>
       <c r="F2">
         <v>0.12</v>
@@ -770,19 +770,19 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3">
-        <v>1344.732986752085</v>
+        <v>1323.581774186526</v>
       </c>
       <c r="B3" t="s">
         <v>30</v>
       </c>
       <c r="C3">
-        <v>1.626629293157687</v>
+        <v>1.672962405293818</v>
       </c>
       <c r="D3">
-        <v>826.6991086467087</v>
+        <v>791.1605006772811</v>
       </c>
       <c r="E3">
-        <v>0.07377218675746983</v>
+        <v>0.07172904759860681</v>
       </c>
       <c r="F3">
         <v>0.12</v>
@@ -790,19 +790,19 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4">
-        <v>40156.76457336248</v>
+        <v>42155.82838774918</v>
       </c>
       <c r="B4" t="s">
         <v>30</v>
       </c>
       <c r="C4">
-        <v>3.168587492581788</v>
+        <v>3.137191306549433</v>
       </c>
       <c r="D4">
-        <v>12673.39616386684</v>
+        <v>13437.44268949794</v>
       </c>
       <c r="E4">
-        <v>0.0378717647156472</v>
+        <v>0.03825077538289715</v>
       </c>
       <c r="F4">
         <v>0.12</v>
@@ -838,693 +838,693 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="7">
-        <v>45866</v>
+        <v>45867</v>
       </c>
       <c r="B2" s="2">
-        <v>54.69454956054688</v>
+        <v>54.96</v>
       </c>
       <c r="C2" s="2">
-        <v>48.44998168945312</v>
+        <v>48.66</v>
       </c>
       <c r="D2" s="2">
-        <v>637.997802734375</v>
+        <v>636.48</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="7">
-        <v>45867</v>
+        <v>45868</v>
       </c>
       <c r="B3" s="2">
-        <v>54.96130752563477</v>
+        <v>54.42</v>
       </c>
       <c r="C3" s="2">
-        <v>48.65766525268555</v>
+        <v>48.5</v>
       </c>
       <c r="D3" s="2">
-        <v>636.482421875</v>
+        <v>635.6</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7">
-        <v>45868</v>
+        <v>45869</v>
       </c>
       <c r="B4" s="2">
-        <v>54.41791915893555</v>
+        <v>54.04</v>
       </c>
       <c r="C4" s="2">
-        <v>48.49942779541016</v>
+        <v>48.6</v>
       </c>
       <c r="D4" s="2">
-        <v>635.5950927734375</v>
+        <v>632.99</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="7">
-        <v>45869</v>
+        <v>45870</v>
       </c>
       <c r="B5" s="2">
-        <v>54.04248428344727</v>
+        <v>53.87</v>
       </c>
       <c r="C5" s="2">
-        <v>48.59832382202149</v>
+        <v>49.04</v>
       </c>
       <c r="D5" s="2">
-        <v>632.992919921875</v>
+        <v>622.77</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="7">
-        <v>45870</v>
+        <v>45873</v>
       </c>
       <c r="B6" s="2">
-        <v>53.87452697753906</v>
+        <v>54.48</v>
       </c>
       <c r="C6" s="2">
-        <v>49.03717041015625</v>
+        <v>49.04</v>
       </c>
       <c r="D6" s="2">
-        <v>622.7737426757812</v>
+        <v>632.27</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="7">
-        <v>45873</v>
+        <v>45874</v>
       </c>
       <c r="B7" s="2">
-        <v>54.47719573974609</v>
+        <v>54.81</v>
       </c>
       <c r="C7" s="2">
-        <v>49.03717041015625</v>
+        <v>49.03</v>
       </c>
       <c r="D7" s="2">
-        <v>632.2650756835938</v>
+        <v>629.22</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="7">
-        <v>45874</v>
+        <v>45875</v>
       </c>
       <c r="B8" s="2">
-        <v>54.81310653686523</v>
+        <v>55.24</v>
       </c>
       <c r="C8" s="2">
-        <v>49.02724075317383</v>
+        <v>48.89</v>
       </c>
       <c r="D8" s="2">
-        <v>629.2242431640625</v>
+        <v>633.88</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="7">
-        <v>45875</v>
+        <v>45876</v>
       </c>
       <c r="B9" s="2">
-        <v>55.23793792724609</v>
+        <v>55.23</v>
       </c>
       <c r="C9" s="2">
-        <v>48.88824462890625</v>
+        <v>48.86</v>
       </c>
       <c r="D9" s="2">
-        <v>633.8801879882812</v>
+        <v>633.53</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="7">
-        <v>45876</v>
+        <v>45877</v>
       </c>
       <c r="B10" s="2">
-        <v>55.22806167602539</v>
+        <v>55.28</v>
       </c>
       <c r="C10" s="2">
-        <v>48.85845565795898</v>
+        <v>48.85</v>
       </c>
       <c r="D10" s="2">
-        <v>633.5313110351562</v>
+        <v>638.33</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="7">
-        <v>45877</v>
+        <v>45880</v>
       </c>
       <c r="B11" s="2">
-        <v>55.27745819091797</v>
+        <v>55.33</v>
       </c>
       <c r="C11" s="2">
-        <v>48.84852600097656</v>
+        <v>48.91</v>
       </c>
       <c r="D11" s="2">
-        <v>638.3268432617188</v>
+        <v>637.0599999999999</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="7">
-        <v>45880</v>
+        <v>45881</v>
       </c>
       <c r="B12" s="2">
-        <v>55.32685852050781</v>
+        <v>55.93</v>
       </c>
       <c r="C12" s="2">
-        <v>48.90809631347656</v>
+        <v>48.98</v>
       </c>
       <c r="D12" s="2">
-        <v>637.0606079101562</v>
+        <v>643.8</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="7">
-        <v>45881</v>
+        <v>45882</v>
       </c>
       <c r="B13" s="2">
-        <v>55.92952346801758</v>
+        <v>56.13</v>
       </c>
       <c r="C13" s="2">
-        <v>48.97759628295898</v>
+        <v>49</v>
       </c>
       <c r="D13" s="2">
-        <v>643.8003540039062</v>
+        <v>646.16</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="7">
-        <v>45882</v>
+        <v>45883</v>
       </c>
       <c r="B14" s="2">
-        <v>56.12712097167969</v>
+        <v>55.68</v>
       </c>
       <c r="C14" s="2">
-        <v>48.99745559692383</v>
+        <v>48.85</v>
       </c>
       <c r="D14" s="2">
-        <v>646.1632080078125</v>
+        <v>646.1799999999999</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="7">
-        <v>45883</v>
+        <v>45884</v>
       </c>
       <c r="B15" s="2">
-        <v>55.68252944946289</v>
+        <v>55.74</v>
       </c>
       <c r="C15" s="2">
-        <v>48.84852600097656</v>
+        <v>48.87</v>
       </c>
       <c r="D15" s="2">
-        <v>646.1831665039062</v>
+        <v>644.73</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="7">
-        <v>45884</v>
+        <v>45887</v>
       </c>
       <c r="B16" s="2">
-        <v>55.74180603027344</v>
+        <v>55.67</v>
       </c>
       <c r="C16" s="2">
-        <v>48.86838531494141</v>
+        <v>48.91</v>
       </c>
       <c r="D16" s="2">
-        <v>644.7275390625</v>
+        <v>644.4299999999999</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="7">
-        <v>45887</v>
+        <v>45888</v>
       </c>
       <c r="B17" s="2">
-        <v>55.67264938354492</v>
+        <v>55.37</v>
       </c>
       <c r="C17" s="2">
-        <v>48.90809631347656</v>
+        <v>48.86</v>
       </c>
       <c r="D17" s="2">
-        <v>644.428466796875</v>
+        <v>641.02</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="7">
-        <v>45888</v>
+        <v>45889</v>
       </c>
       <c r="B18" s="2">
-        <v>55.36637878417969</v>
+        <v>55.53</v>
       </c>
       <c r="C18" s="2">
-        <v>48.85845565795898</v>
+        <v>48.93</v>
       </c>
       <c r="D18" s="2">
-        <v>641.0187377929688</v>
+        <v>639.3</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="7">
-        <v>45889</v>
+        <v>45890</v>
       </c>
       <c r="B19" s="2">
-        <v>55.53433227539063</v>
+        <v>55.79</v>
       </c>
       <c r="C19" s="2">
-        <v>48.92795181274414</v>
+        <v>48.78</v>
       </c>
       <c r="D19" s="2">
-        <v>639.3038940429688</v>
+        <v>636.78</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="7">
-        <v>45890</v>
+        <v>45891</v>
       </c>
       <c r="B20" s="2">
-        <v>55.79121017456055</v>
+        <v>56.65</v>
       </c>
       <c r="C20" s="2">
-        <v>48.77902603149414</v>
+        <v>48.97</v>
       </c>
       <c r="D20" s="2">
-        <v>636.781494140625</v>
+        <v>646.55</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="7">
-        <v>45891</v>
+        <v>45894</v>
       </c>
       <c r="B21" s="2">
-        <v>56.65074920654297</v>
+        <v>55.92</v>
       </c>
       <c r="C21" s="2">
-        <v>48.96766662597656</v>
+        <v>48.91</v>
       </c>
       <c r="D21" s="2">
-        <v>646.5520629882812</v>
+        <v>643.7</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="7">
-        <v>45894</v>
+        <v>45895</v>
       </c>
       <c r="B22" s="2">
-        <v>55.91964340209961</v>
+        <v>56.13</v>
       </c>
       <c r="C22" s="2">
-        <v>48.90809631347656</v>
+        <v>48.98</v>
       </c>
       <c r="D22" s="2">
-        <v>643.70068359375</v>
+        <v>646.3099999999999</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="7">
-        <v>45895</v>
+        <v>45896</v>
       </c>
       <c r="B23" s="2">
-        <v>56.12712097167969</v>
+        <v>56</v>
       </c>
       <c r="C23" s="2">
-        <v>48.97759628295898</v>
+        <v>49.08</v>
       </c>
       <c r="D23" s="2">
-        <v>646.3128051757812</v>
+        <v>647.85</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="7">
-        <v>45896</v>
+        <v>45897</v>
       </c>
       <c r="B24" s="2">
-        <v>55.99868392944336</v>
+        <v>56.25</v>
       </c>
       <c r="C24" s="2">
-        <v>49.07688140869141</v>
+        <v>49.12</v>
       </c>
       <c r="D24" s="2">
-        <v>647.84814453125</v>
+        <v>650.1799999999999</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="7">
-        <v>45897</v>
+        <v>45898</v>
       </c>
       <c r="B25" s="2">
-        <v>56.24567794799805</v>
+        <v>56.24</v>
       </c>
       <c r="C25" s="2">
-        <v>49.11659622192383</v>
+        <v>49.14</v>
       </c>
       <c r="D25" s="2">
-        <v>650.18115234375</v>
+        <v>646.37</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="7">
-        <v>45898</v>
-      </c>
-      <c r="B26" s="2">
-        <v>56.23579788208008</v>
-      </c>
-      <c r="C26" s="2">
-        <v>49.13645935058594</v>
-      </c>
-      <c r="D26" s="2">
-        <v>646.3726196289062</v>
+        <v>45901</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="7">
-        <v>45901</v>
+        <v>45902</v>
+      </c>
+      <c r="B27" s="2">
+        <v>55.84</v>
+      </c>
+      <c r="C27" s="2">
+        <v>49.12</v>
+      </c>
+      <c r="D27" s="2">
+        <v>641.49</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="7">
-        <v>45902</v>
+        <v>45903</v>
       </c>
       <c r="B28" s="2">
-        <v>55.84060668945312</v>
+        <v>55.49</v>
       </c>
       <c r="C28" s="2">
-        <v>49.12150573730469</v>
+        <v>49.31</v>
       </c>
       <c r="D28" s="2">
-        <v>641.4873046875</v>
+        <v>644.9400000000001</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="7">
-        <v>45903</v>
+        <v>45904</v>
       </c>
       <c r="B29" s="2">
-        <v>55.49481201171875</v>
+        <v>55.84</v>
       </c>
       <c r="C29" s="2">
-        <v>49.31085586547852</v>
+        <v>49.49</v>
       </c>
       <c r="D29" s="2">
-        <v>644.9369506835938</v>
+        <v>650.25</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="7">
-        <v>45904</v>
+        <v>45905</v>
       </c>
       <c r="B30" s="2">
-        <v>55.84060668945312</v>
+        <v>56</v>
       </c>
       <c r="C30" s="2">
-        <v>49.49023818969727</v>
+        <v>49.97</v>
       </c>
       <c r="D30" s="2">
-        <v>650.2509155273438</v>
+        <v>648.52</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="7">
-        <v>45905</v>
+        <v>45908</v>
       </c>
       <c r="B31" s="2">
-        <v>55.99868392944336</v>
+        <v>56.29</v>
       </c>
       <c r="C31" s="2">
-        <v>49.96859741210938</v>
+        <v>50.22</v>
       </c>
       <c r="D31" s="2">
-        <v>648.51611328125</v>
+        <v>650.16</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="7">
-        <v>45908</v>
+        <v>45909</v>
       </c>
       <c r="B32" s="2">
-        <v>56.29507827758789</v>
+        <v>56.13</v>
       </c>
       <c r="C32" s="2">
-        <v>50.21774291992188</v>
+        <v>50.23</v>
       </c>
       <c r="D32" s="2">
-        <v>650.1611938476562</v>
+        <v>651.66</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="7">
-        <v>45909</v>
+        <v>45910</v>
       </c>
       <c r="B33" s="2">
-        <v>56.12712097167969</v>
+        <v>56.6</v>
       </c>
       <c r="C33" s="2">
-        <v>50.22771072387695</v>
+        <v>50.49</v>
       </c>
       <c r="D33" s="2">
-        <v>651.6566772460938</v>
+        <v>653.52</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="7">
-        <v>45910</v>
+        <v>45911</v>
       </c>
       <c r="B34" s="2">
-        <v>56.60135269165039</v>
+        <v>57.18</v>
       </c>
       <c r="C34" s="2">
-        <v>50.48682022094727</v>
+        <v>50.63</v>
       </c>
       <c r="D34" s="2">
-        <v>653.5210571289062</v>
+        <v>658.96</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="7">
-        <v>45911</v>
+        <v>45912</v>
       </c>
       <c r="B35" s="2">
-        <v>57.18426132202149</v>
+        <v>56.84</v>
       </c>
       <c r="C35" s="2">
-        <v>50.6263427734375</v>
+        <v>50.56</v>
       </c>
       <c r="D35" s="2">
-        <v>658.9646606445312</v>
+        <v>658.74</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="7">
-        <v>45912</v>
+        <v>45915</v>
       </c>
       <c r="B36" s="2">
-        <v>56.83846282958984</v>
+        <v>57.36</v>
       </c>
       <c r="C36" s="2">
-        <v>50.55658340454102</v>
+        <v>50.7</v>
       </c>
       <c r="D36" s="2">
-        <v>658.7352905273438</v>
+        <v>662.1799999999999</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="7">
-        <v>45915</v>
+        <v>45916</v>
       </c>
       <c r="B37" s="2">
-        <v>57.36209487915039</v>
+        <v>57.04</v>
       </c>
       <c r="C37" s="2">
-        <v>50.69610214233398</v>
+        <v>50.77</v>
       </c>
       <c r="D37" s="2">
-        <v>662.1749877929688</v>
+        <v>661.3</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="7">
-        <v>45916</v>
+        <v>45917</v>
       </c>
       <c r="B38" s="2">
-        <v>57.03606033325195</v>
+        <v>56.65</v>
       </c>
       <c r="C38" s="2">
-        <v>50.76586151123047</v>
+        <v>50.76</v>
       </c>
       <c r="D38" s="2">
-        <v>661.2999877929688</v>
+        <v>660.5700000000001</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="7">
-        <v>45917</v>
+        <v>45918</v>
       </c>
       <c r="B39" s="2">
-        <v>56.65074920654297</v>
+        <v>56.22</v>
       </c>
       <c r="C39" s="2">
-        <v>50.75589752197266</v>
+        <v>50.76</v>
       </c>
       <c r="D39" s="2">
-        <v>660.5700073242188</v>
+        <v>663.7</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="7">
-        <v>45918</v>
+        <v>45919</v>
       </c>
       <c r="B40" s="2">
-        <v>56.21604156494141</v>
+        <v>56.08</v>
       </c>
       <c r="C40" s="2">
-        <v>50.75589752197266</v>
+        <v>50.74</v>
       </c>
       <c r="D40" s="2">
-        <v>663.7000122070312</v>
+        <v>666.87</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="7">
-        <v>45919</v>
+        <v>45922</v>
       </c>
       <c r="B41" s="2">
-        <v>56.07772064208984</v>
+        <v>56.14</v>
       </c>
       <c r="C41" s="2">
-        <v>50.73596572875977</v>
+        <v>50.66</v>
       </c>
       <c r="D41" s="2">
-        <v>666.8699951171875</v>
+        <v>670.08</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="7">
-        <v>45922</v>
+        <v>45923</v>
       </c>
       <c r="B42" s="2">
-        <v>56.13700103759766</v>
+        <v>55.91</v>
       </c>
       <c r="C42" s="2">
-        <v>50.65624237060547</v>
+        <v>50.6</v>
       </c>
       <c r="D42" s="2">
-        <v>670.0800170898438</v>
+        <v>666.5</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="7">
-        <v>45923</v>
+        <v>45924</v>
       </c>
       <c r="B43" s="2">
-        <v>55.90999984741211</v>
+        <v>55.26</v>
       </c>
       <c r="C43" s="2">
-        <v>50.5964469909668</v>
+        <v>50.56</v>
       </c>
       <c r="D43" s="2">
-        <v>666.5</v>
+        <v>664.26</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="7">
-        <v>45924</v>
+        <v>45925</v>
       </c>
       <c r="B44" s="2">
-        <v>55.2599983215332</v>
+        <v>55.19</v>
       </c>
       <c r="C44" s="2">
-        <v>50.55658340454102</v>
+        <v>50.53</v>
       </c>
       <c r="D44" s="2">
-        <v>664.260009765625</v>
+        <v>661.22</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="7">
-        <v>45925</v>
+        <v>45926</v>
       </c>
       <c r="B45" s="2">
-        <v>55.18999862670898</v>
+        <v>55.53</v>
       </c>
       <c r="C45" s="2">
-        <v>50.52668380737305</v>
+        <v>50.52</v>
       </c>
       <c r="D45" s="2">
-        <v>661.219970703125</v>
+        <v>664.89</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="7">
-        <v>45926</v>
+        <v>45929</v>
       </c>
       <c r="B46" s="2">
-        <v>55.52999877929688</v>
+        <v>56.22</v>
       </c>
       <c r="C46" s="2">
-        <v>50.51671600341797</v>
+        <v>50.72</v>
       </c>
       <c r="D46" s="2">
-        <v>664.8900146484375</v>
+        <v>666.76</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="7">
-        <v>45929</v>
+        <v>45930</v>
       </c>
       <c r="B47" s="2">
-        <v>56.22000122070312</v>
+        <v>56.34</v>
       </c>
       <c r="C47" s="2">
-        <v>50.71603393554688</v>
+        <v>50.73</v>
       </c>
       <c r="D47" s="2">
-        <v>666.760009765625</v>
+        <v>669.3</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="7">
-        <v>45930</v>
+        <v>45931</v>
       </c>
       <c r="B48" s="2">
-        <v>56.34000015258789</v>
+        <v>56.66</v>
       </c>
       <c r="C48" s="2">
-        <v>50.72600173950195</v>
+        <v>50.79</v>
       </c>
       <c r="D48" s="2">
-        <v>669.2999877929688</v>
+        <v>671.84</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="7">
-        <v>45931</v>
+        <v>45932</v>
       </c>
       <c r="B49" s="2">
-        <v>56.65999984741211</v>
+        <v>56.78</v>
       </c>
       <c r="C49" s="2">
-        <v>50.79000091552734</v>
+        <v>50.73</v>
       </c>
       <c r="D49" s="2">
-        <v>671.8400268554688</v>
+        <v>672.5</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="7">
-        <v>45932</v>
+        <v>45933</v>
       </c>
       <c r="B50" s="2">
-        <v>56.77999877929688</v>
+        <v>57.13</v>
       </c>
       <c r="C50" s="2">
-        <v>50.72999954223633</v>
+        <v>50.74</v>
       </c>
       <c r="D50" s="2">
-        <v>672.5</v>
+        <v>672.42</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="7">
-        <v>45933</v>
+        <v>45936</v>
       </c>
       <c r="B51" s="2">
-        <v>57.13000106811523</v>
+        <v>57.08</v>
       </c>
       <c r="C51" s="2">
-        <v>50.7400016784668</v>
+        <v>50.64</v>
       </c>
       <c r="D51" s="2">
-        <v>672.4199829101562</v>
+        <v>673.8200000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1557,702 +1557,702 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="7">
-        <v>45866</v>
+        <v>45867</v>
       </c>
       <c r="B2" s="2">
-        <v>0.007328799202481472</v>
+        <v>0.007175035668403553</v>
       </c>
       <c r="C2" s="2">
-        <v>0.002726934919519985</v>
+        <v>0.002898659287325633</v>
       </c>
       <c r="D2" s="2">
-        <v>0.006281532726746747</v>
+        <v>0.0061860895843732</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="7">
-        <v>45867</v>
+        <v>45868</v>
       </c>
       <c r="B3" s="2">
-        <v>0.007175758771914485</v>
+        <v>0.007438738035053693</v>
       </c>
       <c r="C3" s="2">
-        <v>0.002876909061851842</v>
+        <v>0.002903548884727585</v>
       </c>
       <c r="D3" s="2">
-        <v>0.006186184378413733</v>
+        <v>0.006054196772850721</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7">
-        <v>45868</v>
+        <v>45869</v>
       </c>
       <c r="B4" s="2">
-        <v>0.007444470719747479</v>
+        <v>0.007446627838659001</v>
       </c>
       <c r="C4" s="2">
-        <v>0.002880843031622975</v>
+        <v>0.002880489046858354</v>
       </c>
       <c r="D4" s="2">
-        <v>0.006054613662933471</v>
+        <v>0.006027374556314806</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="7">
-        <v>45869</v>
+        <v>45870</v>
       </c>
       <c r="B5" s="2">
-        <v>0.007447271088584301</v>
+        <v>0.00728041630180797</v>
       </c>
       <c r="C5" s="2">
-        <v>0.002857850411468414</v>
+        <v>0.003542848166896667</v>
       </c>
       <c r="D5" s="2">
-        <v>0.006027134009863324</v>
+        <v>0.007112146219982616</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="7">
-        <v>45870</v>
+        <v>45873</v>
       </c>
       <c r="B6" s="2">
-        <v>0.007280140202284538</v>
+        <v>0.007541836954312034</v>
       </c>
       <c r="C6" s="2">
-        <v>0.003522434137955847</v>
+        <v>0.003443440530050618</v>
       </c>
       <c r="D6" s="2">
-        <v>0.007111820498928435</v>
+        <v>0.007741924838701724</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="7">
-        <v>45873</v>
+        <v>45874</v>
       </c>
       <c r="B7" s="2">
-        <v>0.007530267452085643</v>
+        <v>0.007433907202201509</v>
       </c>
       <c r="C7" s="2">
-        <v>0.003423592410895736</v>
+        <v>0.00334784669755384</v>
       </c>
       <c r="D7" s="2">
-        <v>0.00774013209011701</v>
+        <v>0.007647916717073988</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="7">
-        <v>45874</v>
+        <v>45875</v>
       </c>
       <c r="B8" s="2">
-        <v>0.00742723424333216</v>
+        <v>0.007397132975251517</v>
       </c>
       <c r="C8" s="2">
-        <v>0.003328535626657836</v>
+        <v>0.003329756728478964</v>
       </c>
       <c r="D8" s="2">
-        <v>0.007645584398266796</v>
+        <v>0.007591581722480621</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="7">
-        <v>45875</v>
+        <v>45876</v>
       </c>
       <c r="B9" s="2">
-        <v>0.007385960565387101</v>
+        <v>0.007197965339512632</v>
       </c>
       <c r="C9" s="2">
-        <v>0.003310276000971742</v>
+        <v>0.003239327920744699</v>
       </c>
       <c r="D9" s="2">
-        <v>0.007589034303912723</v>
+        <v>0.007387947323844905</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="7">
-        <v>45876</v>
+        <v>45877</v>
       </c>
       <c r="B10" s="2">
-        <v>0.007187064220028369</v>
+        <v>0.006995769290828663</v>
       </c>
       <c r="C10" s="2">
-        <v>0.003220354015378779</v>
+        <v>0.003148379675965413</v>
       </c>
       <c r="D10" s="2">
-        <v>0.007385454134139984</v>
+        <v>0.007339266011093789</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="7">
-        <v>45877</v>
+        <v>45880</v>
       </c>
       <c r="B11" s="2">
-        <v>0.006985202571394566</v>
+        <v>0.006799222782190714</v>
       </c>
       <c r="C11" s="2">
-        <v>0.003129933513937651</v>
+        <v>0.003073454144081334</v>
       </c>
       <c r="D11" s="2">
-        <v>0.00733654787847324</v>
+        <v>0.007175676353321174</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="7">
-        <v>45880</v>
+        <v>45881</v>
       </c>
       <c r="B12" s="2">
-        <v>0.00678897858313052</v>
+        <v>0.006973108475155003</v>
       </c>
       <c r="C12" s="2">
-        <v>0.003055438797708457</v>
+        <v>0.003004137156279772</v>
       </c>
       <c r="D12" s="2">
-        <v>0.00717289455887074</v>
+        <v>0.007305936303616504</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="7">
-        <v>45881</v>
+        <v>45882</v>
       </c>
       <c r="B13" s="2">
-        <v>0.006967556529462191</v>
+        <v>0.006789331624872962</v>
       </c>
       <c r="C13" s="2">
-        <v>0.002986514005042436</v>
+        <v>0.002920245326109886</v>
       </c>
       <c r="D13" s="2">
-        <v>0.007303321189228063</v>
+        <v>0.007114392387676379</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="7">
-        <v>45882</v>
+        <v>45883</v>
       </c>
       <c r="B14" s="2">
-        <v>0.006783348913856569</v>
+        <v>0.006988235334125304</v>
       </c>
       <c r="C14" s="2">
-        <v>0.002903118450069069</v>
+        <v>0.002933843556362592</v>
       </c>
       <c r="D14" s="2">
-        <v>0.007111920461397651</v>
+        <v>0.00692662880049143</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="7">
-        <v>45883</v>
+        <v>45884</v>
       </c>
       <c r="B15" s="2">
-        <v>0.006975215365830901</v>
+        <v>0.006791616818194528</v>
       </c>
       <c r="C15" s="2">
-        <v>0.002916346460235591</v>
+        <v>0.002853080755809537</v>
       </c>
       <c r="D15" s="2">
-        <v>0.006924236147188805</v>
+        <v>0.006794646664632434</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="7">
-        <v>45884</v>
+        <v>45887</v>
       </c>
       <c r="B16" s="2">
-        <v>0.006778998082082067</v>
+        <v>0.00662746170199507</v>
       </c>
       <c r="C16" s="2">
-        <v>0.002836069585509576</v>
+        <v>0.002779427743432645</v>
       </c>
       <c r="D16" s="2">
-        <v>0.006792627529544324</v>
+        <v>0.006619189496223638</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="7">
-        <v>45887</v>
+        <v>45888</v>
       </c>
       <c r="B17" s="2">
-        <v>0.006614968903908455</v>
+        <v>0.006619278519029583</v>
       </c>
       <c r="C17" s="2">
-        <v>0.00276285401566731</v>
+        <v>0.002712226767801876</v>
       </c>
       <c r="D17" s="2">
-        <v>0.006617205367220879</v>
+        <v>0.006618154474301606</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="7">
-        <v>45888</v>
+        <v>45889</v>
       </c>
       <c r="B18" s="2">
-        <v>0.006613691632599773</v>
+        <v>0.006450799941297964</v>
       </c>
       <c r="C18" s="2">
-        <v>0.002696009285830146</v>
+        <v>0.00265751411324298</v>
       </c>
       <c r="D18" s="2">
-        <v>0.006616251402475079</v>
+        <v>0.006489350416626811</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="7">
-        <v>45889</v>
+        <v>45890</v>
       </c>
       <c r="B19" s="2">
-        <v>0.006448041305506382</v>
+        <v>0.006329353627726219</v>
       </c>
       <c r="C19" s="2">
-        <v>0.002641596788151095</v>
+        <v>0.002682554505165646</v>
       </c>
       <c r="D19" s="2">
-        <v>0.006487266282330647</v>
+        <v>0.006403056743962909</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="7">
-        <v>45890</v>
+        <v>45891</v>
       </c>
       <c r="B20" s="2">
-        <v>0.006324761129974907</v>
+        <v>0.006988655841198348</v>
       </c>
       <c r="C20" s="2">
-        <v>0.002666216861700333</v>
+        <v>0.00276879130257831</v>
       </c>
       <c r="D20" s="2">
-        <v>0.006401226441551826</v>
+        <v>0.007108121164210875</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="7">
-        <v>45891</v>
+        <v>45894</v>
       </c>
       <c r="B21" s="2">
-        <v>0.006983667244971634</v>
+        <v>0.007615090771794893</v>
       </c>
       <c r="C21" s="2">
-        <v>0.002751657968203692</v>
+        <v>0.002708479070755818</v>
       </c>
       <c r="D21" s="2">
-        <v>0.007106645446815828</v>
+        <v>0.007037646947425417</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="7">
-        <v>45894</v>
+        <v>45895</v>
       </c>
       <c r="B22" s="2">
-        <v>0.007612853878636079</v>
+        <v>0.007426034213318407</v>
       </c>
       <c r="C22" s="2">
-        <v>0.002691667821314292</v>
+        <v>0.002652209217000748</v>
       </c>
       <c r="D22" s="2">
-        <v>0.007036341161346941</v>
+        <v>0.006874700102781585</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="7">
-        <v>45895</v>
+        <v>45896</v>
       </c>
       <c r="B23" s="2">
-        <v>0.00742301913947778</v>
+        <v>0.007264420558885818</v>
       </c>
       <c r="C23" s="2">
-        <v>0.002635730169523902</v>
+        <v>0.002616337535021625</v>
       </c>
       <c r="D23" s="2">
-        <v>0.006873514069976145</v>
+        <v>0.006686416776200166</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="7">
-        <v>45896</v>
+        <v>45897</v>
       </c>
       <c r="B24" s="2">
-        <v>0.007260694107083811</v>
+        <v>0.007103985799218884</v>
       </c>
       <c r="C24" s="2">
-        <v>0.002600037837180606</v>
+        <v>0.002546429556859194</v>
       </c>
       <c r="D24" s="2">
-        <v>0.006685195695414147</v>
+        <v>0.006520101593862157</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="7">
-        <v>45897</v>
+        <v>45898</v>
       </c>
       <c r="B25" s="2">
-        <v>0.007099044791044708</v>
+        <v>0.006911775564915628</v>
       </c>
       <c r="C25" s="2">
-        <v>0.002530566580711072</v>
+        <v>0.002474956342874467</v>
       </c>
       <c r="D25" s="2">
-        <v>0.006519011538169736</v>
+        <v>0.006558277917903807</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="7">
-        <v>45898</v>
+        <v>45901</v>
       </c>
       <c r="B26" s="2">
-        <v>0.006906908147926689</v>
+        <v>0.006722524515137882</v>
       </c>
       <c r="C26" s="2">
-        <v>0.002459540502375734</v>
+        <v>0.002405973419147194</v>
       </c>
       <c r="D26" s="2">
-        <v>0.006557123401211668</v>
+        <v>0.006377854147946721</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="7">
-        <v>45901</v>
+        <v>45902</v>
       </c>
       <c r="B27" s="2">
-        <v>0.006717761308806733</v>
+        <v>0.006806428670504493</v>
       </c>
       <c r="C27" s="2">
-        <v>0.002390982968538602</v>
+        <v>0.002343072936032648</v>
       </c>
       <c r="D27" s="2">
-        <v>0.006376734666880324</v>
+        <v>0.006505868767052582</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="7">
-        <v>45902</v>
+        <v>45903</v>
       </c>
       <c r="B28" s="2">
-        <v>0.006796228713279781</v>
+        <v>0.006807083461329025</v>
       </c>
       <c r="C28" s="2">
-        <v>0.002327079107289293</v>
+        <v>0.002430778592175304</v>
       </c>
       <c r="D28" s="2">
-        <v>0.006505424776903935</v>
+        <v>0.006424027451137088</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="7">
-        <v>45903</v>
+        <v>45904</v>
       </c>
       <c r="B29" s="2">
-        <v>0.006793397600206941</v>
+        <v>0.006762809709318349</v>
       </c>
       <c r="C29" s="2">
-        <v>0.002414839717810367</v>
+        <v>0.002479354748707878</v>
       </c>
       <c r="D29" s="2">
-        <v>0.006423592293644437</v>
+        <v>0.006480334449643642</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="7">
-        <v>45904</v>
+        <v>45905</v>
       </c>
       <c r="B30" s="2">
-        <v>0.006745875484655802</v>
+        <v>0.006593347583062813</v>
       </c>
       <c r="C30" s="2">
-        <v>0.002463520018906141</v>
+        <v>0.003207221253091436</v>
       </c>
       <c r="D30" s="2">
-        <v>0.006480330723468721</v>
+        <v>0.006360429796150112</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="7">
-        <v>45905</v>
+        <v>45908</v>
       </c>
       <c r="B31" s="2">
-        <v>0.006576291774884866</v>
+        <v>0.006490655086667903</v>
       </c>
       <c r="C31" s="2">
-        <v>0.003190291266782094</v>
+        <v>0.003246363577416538</v>
       </c>
       <c r="D31" s="2">
-        <v>0.00636066900093449</v>
+        <v>0.00619198228354119</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="7">
-        <v>45908</v>
+        <v>45909</v>
       </c>
       <c r="B32" s="2">
-        <v>0.006478637038875456</v>
+        <v>0.006369773046936044</v>
       </c>
       <c r="C32" s="2">
-        <v>0.003229473042591894</v>
+        <v>0.00316551976781321</v>
       </c>
       <c r="D32" s="2">
-        <v>0.006192326799900102</v>
+        <v>0.006024654615825902</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="7">
-        <v>45909</v>
+        <v>45910</v>
       </c>
       <c r="B33" s="2">
-        <v>0.006363038967097874</v>
+        <v>0.006438212480107756</v>
       </c>
       <c r="C33" s="2">
-        <v>0.003149152277165528</v>
+        <v>0.003208668314316392</v>
       </c>
       <c r="D33" s="2">
-        <v>0.00602490941768656</v>
+        <v>0.005868825848007094</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="7">
-        <v>45910</v>
+        <v>45911</v>
       </c>
       <c r="B34" s="2">
-        <v>0.006436975645191595</v>
+        <v>0.006601929934246859</v>
       </c>
       <c r="C34" s="2">
-        <v>0.003192331104537283</v>
+        <v>0.003132929661823564</v>
       </c>
       <c r="D34" s="2">
-        <v>0.005869185313540195</v>
+        <v>0.005938095116820036</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="7">
-        <v>45911</v>
+        <v>45912</v>
       </c>
       <c r="B35" s="2">
-        <v>0.006604481802921286</v>
+        <v>0.006656635039186004</v>
       </c>
       <c r="C35" s="2">
-        <v>0.00311696242445413</v>
+        <v>0.003119626292072098</v>
       </c>
       <c r="D35" s="2">
-        <v>0.005938779447805829</v>
+        <v>0.005788411206750003</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="7">
-        <v>45912</v>
+        <v>45915</v>
       </c>
       <c r="B36" s="2">
-        <v>0.006665581026876101</v>
+        <v>0.006723685883108747</v>
       </c>
       <c r="C36" s="2">
-        <v>0.003104127215423213</v>
+        <v>0.003048870934067467</v>
       </c>
       <c r="D36" s="2">
-        <v>0.005789340220697785</v>
+        <v>0.005691441642261892</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="7">
-        <v>45915</v>
+        <v>45916</v>
       </c>
       <c r="B37" s="2">
-        <v>0.006736226108240596</v>
+        <v>0.006749709785775677</v>
       </c>
       <c r="C37" s="2">
-        <v>0.003033712031997523</v>
+        <v>0.002963023195828201</v>
       </c>
       <c r="D37" s="2">
-        <v>0.005692333328344287</v>
+        <v>0.005575905597909902</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="7">
-        <v>45916</v>
+        <v>45917</v>
       </c>
       <c r="B38" s="2">
-        <v>0.006767776963877583</v>
+        <v>0.006826475002557245</v>
       </c>
       <c r="C38" s="2">
-        <v>0.002948294870881609</v>
+        <v>0.002904956492103213</v>
       </c>
       <c r="D38" s="2">
-        <v>0.00557653188443315</v>
+        <v>0.005453486456824512</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="7">
-        <v>45917</v>
+        <v>45918</v>
       </c>
       <c r="B39" s="2">
-        <v>0.006837878650127275</v>
+        <v>0.006917706978921328</v>
       </c>
       <c r="C39" s="2">
-        <v>0.002890670509034807</v>
+        <v>0.002840779529520517</v>
       </c>
       <c r="D39" s="2">
-        <v>0.005454091423531432</v>
+        <v>0.005356611283609919</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="7">
-        <v>45918</v>
+        <v>45919</v>
       </c>
       <c r="B40" s="2">
-        <v>0.006933876246341317</v>
+        <v>0.006755719347640018</v>
       </c>
       <c r="C40" s="2">
-        <v>0.002826922371794778</v>
+        <v>0.002788200550149779</v>
       </c>
       <c r="D40" s="2">
-        <v>0.005357191988205764</v>
+        <v>0.005258507696246811</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="7">
-        <v>45919</v>
+        <v>45922</v>
       </c>
       <c r="B41" s="2">
-        <v>0.006770595737751711</v>
+        <v>0.006568373497699827</v>
       </c>
       <c r="C41" s="2">
-        <v>0.002774752470093232</v>
+        <v>0.002785009960949386</v>
       </c>
       <c r="D41" s="2">
-        <v>0.005259064374770869</v>
+        <v>0.005159545827071705</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="7">
-        <v>45922</v>
+        <v>45923</v>
       </c>
       <c r="B42" s="2">
-        <v>0.006582748599095168</v>
+        <v>0.006463268993917766</v>
       </c>
       <c r="C42" s="2">
-        <v>0.002771901183695003</v>
+        <v>0.00275540236883963</v>
       </c>
       <c r="D42" s="2">
-        <v>0.005160081708723377</v>
+        <v>0.005291016468355511</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="7">
-        <v>45923</v>
+        <v>45924</v>
       </c>
       <c r="B43" s="2">
-        <v>0.006475052622496149</v>
+        <v>0.006839641342784614</v>
       </c>
       <c r="C43" s="2">
-        <v>0.002742647376477667</v>
+        <v>0.002706944880655515</v>
       </c>
       <c r="D43" s="2">
-        <v>0.005291514235789576</v>
+        <v>0.005265640369001033</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="7">
-        <v>45924</v>
+        <v>45925</v>
       </c>
       <c r="B44" s="2">
-        <v>0.006850214013124958</v>
+        <v>0.006648607780599038</v>
       </c>
       <c r="C44" s="2">
-        <v>0.002694549357022956</v>
+        <v>0.002651110697157777</v>
       </c>
       <c r="D44" s="2">
-        <v>0.00526611344203308</v>
+        <v>0.005293414409701097</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="7">
-        <v>45925</v>
+        <v>45926</v>
       </c>
       <c r="B45" s="2">
-        <v>0.006658882741892209</v>
+        <v>0.006652937396128402</v>
       </c>
       <c r="C45" s="2">
-        <v>0.00263907056213464</v>
+        <v>0.002585653379337949</v>
       </c>
       <c r="D45" s="2">
-        <v>0.005293863997601853</v>
+        <v>0.005255322730751563</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="7">
-        <v>45926</v>
+        <v>45929</v>
       </c>
       <c r="B46" s="2">
-        <v>0.006662607886116978</v>
+        <v>0.007108084148991159</v>
       </c>
       <c r="C46" s="2">
-        <v>0.002573964408936609</v>
+        <v>0.002625167371784854</v>
       </c>
       <c r="D46" s="2">
-        <v>0.005255752500979861</v>
+        <v>0.005121272932570073</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="7">
-        <v>45929</v>
+        <v>45930</v>
       </c>
       <c r="B47" s="2">
-        <v>0.007116591914784447</v>
+        <v>0.006919245175568222</v>
       </c>
       <c r="C47" s="2">
-        <v>0.00261345802391646</v>
+        <v>0.002556007512588961</v>
       </c>
       <c r="D47" s="2">
-        <v>0.005121688888321384</v>
+        <v>0.00501175115942522</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="7">
-        <v>45930</v>
+        <v>45931</v>
       </c>
       <c r="B48" s="2">
-        <v>0.006927493304865751</v>
+        <v>0.006830427334775744</v>
       </c>
       <c r="C48" s="2">
-        <v>0.002544636864391275</v>
+        <v>0.002485317249367855</v>
       </c>
       <c r="D48" s="2">
-        <v>0.005012151046706876</v>
+        <v>0.004901864211570783</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="7">
-        <v>45931</v>
+        <v>45932</v>
       </c>
       <c r="B49" s="2">
-        <v>0.006838301063335362</v>
+        <v>0.006644983676719484</v>
       </c>
       <c r="C49" s="2">
-        <v>0.002474955904123944</v>
+        <v>0.00246113559879186</v>
       </c>
       <c r="D49" s="2">
-        <v>0.004902251347305733</v>
+        <v>0.004765561817748655</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="7">
-        <v>45932</v>
+        <v>45933</v>
       </c>
       <c r="B50" s="2">
-        <v>0.006652623023092131</v>
+        <v>0.006573556377314132</v>
       </c>
       <c r="C50" s="2">
-        <v>0.002451390666129219</v>
+        <v>0.002395119625548508</v>
       </c>
       <c r="D50" s="2">
-        <v>0.004765938303420128</v>
+        <v>0.004646845450298135</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="7">
-        <v>45933</v>
+        <v>45936</v>
       </c>
       <c r="B51" s="2">
-        <v>0.006580835163442976</v>
+        <v>0.006406045445478905</v>
       </c>
       <c r="C51" s="2">
-        <v>0.002385696932113174</v>
+        <v>0.002409572359965174</v>
       </c>
       <c r="D51" s="2">
-        <v>0.004647210948420895</v>
+        <v>0.004518505279176866</v>
       </c>
     </row>
   </sheetData>
@@ -2285,252 +2285,252 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="7">
-        <v>45866</v>
+        <v>45867</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="7">
-        <v>45867</v>
+        <v>45868</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7">
-        <v>45868</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="7">
-        <v>45869</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="7">
-        <v>45870</v>
+        <v>45873</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="7">
-        <v>45873</v>
+        <v>45874</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="7">
-        <v>45874</v>
+        <v>45875</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="7">
-        <v>45875</v>
+        <v>45876</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="7">
-        <v>45876</v>
+        <v>45877</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="7">
-        <v>45877</v>
+        <v>45880</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="7">
-        <v>45880</v>
+        <v>45881</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="7">
-        <v>45881</v>
+        <v>45882</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="7">
-        <v>45882</v>
+        <v>45883</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="7">
-        <v>45883</v>
+        <v>45884</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="7">
-        <v>45884</v>
+        <v>45887</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="7">
-        <v>45887</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="7">
-        <v>45888</v>
+        <v>45889</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="7">
-        <v>45889</v>
+        <v>45890</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="7">
-        <v>45890</v>
+        <v>45891</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="7">
-        <v>45891</v>
+        <v>45894</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="7">
-        <v>45894</v>
+        <v>45895</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" s="7">
-        <v>45895</v>
+        <v>45896</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" s="7">
-        <v>45896</v>
+        <v>45897</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" s="7">
-        <v>45897</v>
+        <v>45898</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" s="7">
-        <v>45898</v>
+        <v>45901</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" s="7">
-        <v>45901</v>
+        <v>45902</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" s="7">
-        <v>45902</v>
+        <v>45903</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" s="7">
-        <v>45903</v>
+        <v>45904</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" s="7">
-        <v>45904</v>
+        <v>45905</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" s="7">
-        <v>45905</v>
+        <v>45908</v>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" s="7">
-        <v>45908</v>
+        <v>45909</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" s="7">
-        <v>45909</v>
+        <v>45910</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" s="7">
-        <v>45910</v>
+        <v>45911</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" s="7">
-        <v>45911</v>
+        <v>45912</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" s="7">
-        <v>45912</v>
+        <v>45915</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" s="7">
-        <v>45915</v>
+        <v>45916</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" s="7">
-        <v>45916</v>
+        <v>45917</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" s="7">
-        <v>45917</v>
+        <v>45918</v>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" s="7">
-        <v>45918</v>
+        <v>45919</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" s="7">
-        <v>45919</v>
+        <v>45922</v>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" s="7">
-        <v>45922</v>
+        <v>45923</v>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" s="7">
-        <v>45923</v>
+        <v>45924</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" s="7">
-        <v>45924</v>
+        <v>45925</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" s="7">
-        <v>45925</v>
+        <v>45926</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" s="7">
-        <v>45926</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" s="7">
-        <v>45929</v>
+        <v>45930</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" s="7">
-        <v>45930</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" s="7">
-        <v>45931</v>
+        <v>45932</v>
       </c>
     </row>
     <row r="50" spans="1:1">
       <c r="A50" s="7">
-        <v>45932</v>
+        <v>45933</v>
       </c>
     </row>
     <row r="51" spans="1:1">
       <c r="A51" s="7">
-        <v>45933</v>
+        <v>45936</v>
       </c>
     </row>
   </sheetData>
@@ -2563,702 +2563,702 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="7">
-        <v>45866</v>
+        <v>45867</v>
       </c>
       <c r="B2" s="2">
-        <v>1.031449934884971</v>
+        <v>1.053554269210551</v>
       </c>
       <c r="C2" s="2">
-        <v>2.772082826793382</v>
+        <v>2.607857188748427</v>
       </c>
       <c r="D2" s="2">
-        <v>1.203414801613166</v>
+        <v>1.221981892936082</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="7">
-        <v>45867</v>
+        <v>45868</v>
       </c>
       <c r="B3" s="2">
-        <v>1.053448102209229</v>
+        <v>1.016205897366297</v>
       </c>
       <c r="C3" s="2">
-        <v>2.627573307902438</v>
+        <v>2.603465538309257</v>
       </c>
       <c r="D3" s="2">
-        <v>1.221963167887813</v>
+        <v>1.248603199367952</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7">
-        <v>45868</v>
+        <v>45869</v>
       </c>
       <c r="B4" s="2">
-        <v>1.015423358457505</v>
+        <v>1.015129213379063</v>
       </c>
       <c r="C4" s="2">
-        <v>2.623985193641696</v>
+        <v>2.624307656517282</v>
       </c>
       <c r="D4" s="2">
-        <v>1.248517226864985</v>
+        <v>1.254159566417649</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="7">
-        <v>45869</v>
+        <v>45870</v>
       </c>
       <c r="B5" s="2">
-        <v>1.015041532699401</v>
+        <v>1.038304562104137</v>
       </c>
       <c r="C5" s="2">
-        <v>2.645096268807312</v>
+        <v>2.133675817895987</v>
       </c>
       <c r="D5" s="2">
-        <v>1.254209620661141</v>
+        <v>1.062870366605458</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="7">
-        <v>45870</v>
+        <v>45873</v>
       </c>
       <c r="B6" s="2">
-        <v>1.038343939834072</v>
+        <v>1.002314092173861</v>
       </c>
       <c r="C6" s="2">
-        <v>2.146041391868687</v>
+        <v>2.195272255819508</v>
       </c>
       <c r="D6" s="2">
-        <v>1.062919046019726</v>
+        <v>0.9764095645046579</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="7">
-        <v>45873</v>
+        <v>45874</v>
       </c>
       <c r="B7" s="2">
-        <v>1.003854047453635</v>
+        <v>1.016866266227523</v>
       </c>
       <c r="C7" s="2">
-        <v>2.207999245507954</v>
+        <v>2.257955678110311</v>
       </c>
       <c r="D7" s="2">
-        <v>0.9766357178628288</v>
+        <v>0.9884115818505732</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="7">
-        <v>45874</v>
+        <v>45875</v>
       </c>
       <c r="B8" s="2">
-        <v>1.017779864284062</v>
+        <v>1.021921531690123</v>
       </c>
       <c r="C8" s="2">
-        <v>2.271055595632841</v>
+        <v>2.270222744962402</v>
       </c>
       <c r="D8" s="2">
-        <v>0.9887131011068541</v>
+        <v>0.9957463064382944</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="7">
-        <v>45875</v>
+        <v>45876</v>
       </c>
       <c r="B9" s="2">
-        <v>1.023467346361111</v>
+        <v>1.050198091214534</v>
       </c>
       <c r="C9" s="2">
-        <v>2.283582836586886</v>
+        <v>2.333598093535006</v>
       </c>
       <c r="D9" s="2">
-        <v>0.9960805495749514</v>
+        <v>1.023192116677203</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="7">
-        <v>45876</v>
+        <v>45877</v>
       </c>
       <c r="B10" s="2">
-        <v>1.051790999601602</v>
+        <v>1.080551565657639</v>
       </c>
       <c r="C10" s="2">
-        <v>2.347347348796191</v>
+        <v>2.401009483669271</v>
       </c>
       <c r="D10" s="2">
-        <v>1.023537526993904</v>
+        <v>1.029978944591758</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="7">
-        <v>45877</v>
+        <v>45880</v>
       </c>
       <c r="B11" s="2">
-        <v>1.082186147491405</v>
+        <v>1.111787288391944</v>
       </c>
       <c r="C11" s="2">
-        <v>2.415159755478157</v>
+        <v>2.459541969982455</v>
       </c>
       <c r="D11" s="2">
-        <v>1.030360543596379</v>
+        <v>1.05346020193425</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="7">
-        <v>45880</v>
+        <v>45881</v>
       </c>
       <c r="B12" s="2">
-        <v>1.113464914879555</v>
+        <v>1.084063081352898</v>
       </c>
       <c r="C12" s="2">
-        <v>2.47404381519732</v>
+        <v>2.516293054191217</v>
       </c>
       <c r="D12" s="2">
-        <v>1.053868755234377</v>
+        <v>1.034677712210908</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="7">
-        <v>45881</v>
+        <v>45882</v>
       </c>
       <c r="B13" s="2">
-        <v>1.084926893412378</v>
+        <v>1.113407015278325</v>
       </c>
       <c r="C13" s="2">
-        <v>2.531141473778936</v>
+        <v>2.588580278717342</v>
       </c>
       <c r="D13" s="2">
-        <v>1.035048201266845</v>
+        <v>1.062534795421014</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="7">
-        <v>45882</v>
+        <v>45883</v>
       </c>
       <c r="B14" s="2">
-        <v>1.11438900699077</v>
+        <v>1.081716499052434</v>
       </c>
       <c r="C14" s="2">
-        <v>2.603851544536427</v>
+        <v>2.576582327912748</v>
       </c>
       <c r="D14" s="2">
-        <v>1.062904106030873</v>
+        <v>1.091337456923955</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="7">
-        <v>45883</v>
+        <v>45884</v>
       </c>
       <c r="B15" s="2">
-        <v>1.083735635922414</v>
+        <v>1.11303238426724</v>
       </c>
       <c r="C15" s="2">
-        <v>2.592040953726013</v>
+        <v>2.649518225094776</v>
       </c>
       <c r="D15" s="2">
-        <v>1.091714565981919</v>
+        <v>1.112536064536253</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="7">
-        <v>45884</v>
+        <v>45887</v>
       </c>
       <c r="B16" s="2">
-        <v>1.115104233495051</v>
+        <v>1.140601002327779</v>
       </c>
       <c r="C16" s="2">
-        <v>2.665410432384125</v>
+        <v>2.719728720433898</v>
       </c>
       <c r="D16" s="2">
-        <v>1.112866770230761</v>
+        <v>1.142026446666506</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="7">
-        <v>45887</v>
+        <v>45888</v>
       </c>
       <c r="B17" s="2">
-        <v>1.142755101345698</v>
+        <v>1.142011087530544</v>
       </c>
       <c r="C17" s="2">
-        <v>2.736043749441012</v>
+        <v>2.787115572312919</v>
       </c>
       <c r="D17" s="2">
-        <v>1.142368876388572</v>
+        <v>1.142205049691327</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="7">
-        <v>45888</v>
+        <v>45889</v>
       </c>
       <c r="B18" s="2">
-        <v>1.142975796289593</v>
+        <v>1.171837528519531</v>
       </c>
       <c r="C18" s="2">
-        <v>2.803881091921727</v>
+        <v>2.844496449714015</v>
       </c>
       <c r="D18" s="2">
-        <v>1.142533588937791</v>
+        <v>1.164876139346146</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="7">
-        <v>45889</v>
+        <v>45890</v>
       </c>
       <c r="B19" s="2">
-        <v>1.172338870368153</v>
+        <v>1.194322501917178</v>
       </c>
       <c r="C19" s="2">
-        <v>2.861636376184209</v>
+        <v>2.817944405464285</v>
       </c>
       <c r="D19" s="2">
-        <v>1.165250373762792</v>
+        <v>1.180575116300786</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="7">
-        <v>45890</v>
+        <v>45891</v>
       </c>
       <c r="B20" s="2">
-        <v>1.195189716234317</v>
+        <v>1.081651412224693</v>
       </c>
       <c r="C20" s="2">
-        <v>2.835211782196794</v>
+        <v>2.730176685091904</v>
       </c>
       <c r="D20" s="2">
-        <v>1.180912678094852</v>
+        <v>1.063472229236227</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="7">
-        <v>45891</v>
+        <v>45894</v>
       </c>
       <c r="B21" s="2">
-        <v>1.082424061030022</v>
+        <v>0.9926722722968675</v>
       </c>
       <c r="C21" s="2">
-        <v>2.747176265195241</v>
+        <v>2.79097207794745</v>
       </c>
       <c r="D21" s="2">
-        <v>1.063693062606849</v>
+        <v>1.074121722310887</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="7">
-        <v>45894</v>
+        <v>45895</v>
       </c>
       <c r="B22" s="2">
-        <v>0.9929639502733854</v>
+        <v>1.017944335164407</v>
       </c>
       <c r="C22" s="2">
-        <v>2.808403548285346</v>
+        <v>2.850185955063142</v>
       </c>
       <c r="D22" s="2">
-        <v>1.074321055054911</v>
+        <v>1.099580977667079</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="7">
-        <v>45895</v>
+        <v>45896</v>
       </c>
       <c r="B23" s="2">
-        <v>1.018357802687324</v>
+        <v>1.040590835691368</v>
       </c>
       <c r="C23" s="2">
-        <v>2.868005817738921</v>
+        <v>2.889263850324291</v>
       </c>
       <c r="D23" s="2">
-        <v>1.099770711636992</v>
+        <v>1.130544163368833</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="7">
-        <v>45896</v>
+        <v>45897</v>
       </c>
       <c r="B24" s="2">
-        <v>1.041124904684996</v>
+        <v>1.064091296609253</v>
       </c>
       <c r="C24" s="2">
-        <v>2.907376712787221</v>
+        <v>2.96858377245208</v>
       </c>
       <c r="D24" s="2">
-        <v>1.130750662298487</v>
+        <v>1.159382158600205</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="7">
-        <v>45897</v>
+        <v>45898</v>
       </c>
       <c r="B25" s="2">
-        <v>1.064831915093764</v>
+        <v>1.093682714258795</v>
       </c>
       <c r="C25" s="2">
-        <v>2.987192480057345</v>
+        <v>3.054312243506091</v>
       </c>
       <c r="D25" s="2">
-        <v>1.159576020984751</v>
+        <v>1.152633291057706</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="7">
-        <v>45898</v>
+        <v>45901</v>
       </c>
       <c r="B26" s="2">
-        <v>1.09445345128177</v>
+        <v>1.124471832443664</v>
       </c>
       <c r="C26" s="2">
-        <v>3.073455978010051</v>
+        <v>3.141884029152725</v>
       </c>
       <c r="D26" s="2">
-        <v>1.152836235899982</v>
+        <v>1.185240252415959</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="7">
-        <v>45901</v>
+        <v>45902</v>
       </c>
       <c r="B27" s="2">
-        <v>1.125269135459547</v>
+        <v>1.110610251884745</v>
       </c>
       <c r="C27" s="2">
-        <v>3.161582311397589</v>
+        <v>3.226228831350052</v>
       </c>
       <c r="D27" s="2">
-        <v>1.185448329761345</v>
+        <v>1.161918527847773</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="7">
-        <v>45902</v>
+        <v>45903</v>
       </c>
       <c r="B28" s="2">
-        <v>1.112277084703425</v>
+        <v>1.110503419434886</v>
       </c>
       <c r="C28" s="2">
-        <v>3.248402444294217</v>
+        <v>3.10982229501196</v>
       </c>
       <c r="D28" s="2">
-        <v>1.161997827877761</v>
+        <v>1.1767212263152</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="7">
-        <v>45903</v>
+        <v>45904</v>
       </c>
       <c r="B29" s="2">
-        <v>1.112740620386222</v>
+        <v>1.117773497274179</v>
       </c>
       <c r="C29" s="2">
-        <v>3.130348322678268</v>
+        <v>3.048893856001883</v>
       </c>
       <c r="D29" s="2">
-        <v>1.176800941688621</v>
+        <v>1.166496809528131</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="7">
-        <v>45904</v>
+        <v>45905</v>
       </c>
       <c r="B30" s="2">
-        <v>1.12057945293816</v>
+        <v>1.146502495879797</v>
       </c>
       <c r="C30" s="2">
-        <v>3.068491184228753</v>
+        <v>2.356959144274239</v>
       </c>
       <c r="D30" s="2">
-        <v>1.166497480261052</v>
+        <v>1.188487209584498</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="7">
-        <v>45905</v>
+        <v>45908</v>
       </c>
       <c r="B31" s="2">
-        <v>1.149475984179076</v>
+        <v>1.164641990561425</v>
       </c>
       <c r="C31" s="2">
-        <v>2.369466869339885</v>
+        <v>2.328540620887646</v>
       </c>
       <c r="D31" s="2">
-        <v>1.188442514313189</v>
+        <v>1.220818974285145</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="7">
-        <v>45908</v>
+        <v>45909</v>
       </c>
       <c r="B32" s="2">
-        <v>1.166802433108163</v>
+        <v>1.186743923917458</v>
       </c>
       <c r="C32" s="2">
-        <v>2.340719170121218</v>
+        <v>2.388008925752695</v>
       </c>
       <c r="D32" s="2">
-        <v>1.220751052787862</v>
+        <v>1.254725779686586</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="7">
-        <v>45909</v>
+        <v>45910</v>
       </c>
       <c r="B33" s="2">
-        <v>1.1879998691305</v>
+        <v>1.174128608451585</v>
       </c>
       <c r="C33" s="2">
-        <v>2.400420429014143</v>
+        <v>2.355896191094795</v>
       </c>
       <c r="D33" s="2">
-        <v>1.254672715575391</v>
+        <v>1.288041195284656</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="7">
-        <v>45910</v>
+        <v>45911</v>
       </c>
       <c r="B34" s="2">
-        <v>1.174354211799965</v>
+        <v>1.145012070026899</v>
       </c>
       <c r="C34" s="2">
-        <v>2.367952825895933</v>
+        <v>2.412850040107366</v>
       </c>
       <c r="D34" s="2">
-        <v>1.287962307604308</v>
+        <v>1.273015893391868</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="7">
-        <v>45911</v>
+        <v>45912</v>
       </c>
       <c r="B35" s="2">
-        <v>1.144569655236377</v>
+        <v>1.135602209777888</v>
       </c>
       <c r="C35" s="2">
-        <v>2.425210326848388</v>
+        <v>2.423139425191715</v>
       </c>
       <c r="D35" s="2">
-        <v>1.272869202606512</v>
+        <v>1.305935115903562</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="7">
-        <v>45912</v>
+        <v>45915</v>
       </c>
       <c r="B36" s="2">
-        <v>1.134078099074176</v>
+        <v>1.124277604814199</v>
       </c>
       <c r="C36" s="2">
-        <v>2.435238292627101</v>
+        <v>2.479373388921969</v>
       </c>
       <c r="D36" s="2">
-        <v>1.305725552828786</v>
+        <v>1.328185358882171</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="7">
-        <v>45915</v>
+        <v>45916</v>
       </c>
       <c r="B37" s="2">
-        <v>1.122184638508062</v>
+        <v>1.119942886450462</v>
       </c>
       <c r="C37" s="2">
-        <v>2.491762362562537</v>
+        <v>2.551208330338984</v>
       </c>
       <c r="D37" s="2">
-        <v>1.327977302830102</v>
+        <v>1.35570614090348</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="7">
-        <v>45916</v>
+        <v>45917</v>
       </c>
       <c r="B38" s="2">
-        <v>1.116953100040322</v>
+        <v>1.10734888172194</v>
       </c>
       <c r="C38" s="2">
-        <v>2.563952993590543</v>
+        <v>2.602204019486555</v>
       </c>
       <c r="D38" s="2">
-        <v>1.355553884895063</v>
+        <v>1.386138852646241</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="7">
-        <v>45917</v>
+        <v>45918</v>
       </c>
       <c r="B39" s="2">
-        <v>1.105502136988617</v>
+        <v>1.092744963499922</v>
       </c>
       <c r="C39" s="2">
-        <v>2.615064372282466</v>
+        <v>2.660991246110691</v>
       </c>
       <c r="D39" s="2">
-        <v>1.385985102407769</v>
+        <v>1.411207395861325</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="7">
-        <v>45918</v>
+        <v>45919</v>
       </c>
       <c r="B40" s="2">
-        <v>1.090196766083506</v>
+        <v>1.118946639313138</v>
       </c>
       <c r="C40" s="2">
-        <v>2.674035033860957</v>
+        <v>2.711171353788904</v>
       </c>
       <c r="D40" s="2">
-        <v>1.411054424935088</v>
+        <v>1.437535113922128</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="7">
-        <v>45919</v>
+        <v>45922</v>
       </c>
       <c r="B41" s="2">
-        <v>1.116488083616514</v>
+        <v>1.150861695491544</v>
       </c>
       <c r="C41" s="2">
-        <v>2.724311282415238</v>
+        <v>2.714277351312469</v>
       </c>
       <c r="D41" s="2">
-        <v>1.437382949037184</v>
+        <v>1.465107533403732</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="7">
-        <v>45922</v>
+        <v>45923</v>
       </c>
       <c r="B42" s="2">
-        <v>1.148348497043257</v>
+        <v>1.169576798876572</v>
       </c>
       <c r="C42" s="2">
-        <v>2.727113615972359</v>
+        <v>2.743443043263389</v>
       </c>
       <c r="D42" s="2">
-        <v>1.464955379951675</v>
+        <v>1.428702689813028</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="7">
-        <v>45923</v>
+        <v>45924</v>
       </c>
       <c r="B43" s="2">
-        <v>1.167448343805184</v>
+        <v>1.105217230163554</v>
       </c>
       <c r="C43" s="2">
-        <v>2.756201735963887</v>
+        <v>2.792553891364786</v>
       </c>
       <c r="D43" s="2">
-        <v>1.428568293184716</v>
+        <v>1.435587873544552</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="7">
-        <v>45924</v>
+        <v>45925</v>
       </c>
       <c r="B44" s="2">
-        <v>1.103511429818251</v>
+        <v>1.136973289692756</v>
       </c>
       <c r="C44" s="2">
-        <v>2.80540025755414</v>
+        <v>2.851366964151578</v>
       </c>
       <c r="D44" s="2">
-        <v>1.435458909762138</v>
+        <v>1.428055480850099</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="7">
-        <v>45925</v>
+        <v>45926</v>
       </c>
       <c r="B45" s="2">
-        <v>1.135218887791448</v>
+        <v>1.136233367321866</v>
       </c>
       <c r="C45" s="2">
-        <v>2.864375651278582</v>
+        <v>2.923550975776994</v>
       </c>
       <c r="D45" s="2">
-        <v>1.427934201484764</v>
+        <v>1.438406325828726</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="7">
-        <v>45926</v>
+        <v>45929</v>
       </c>
       <c r="B46" s="2">
-        <v>1.13458417325384</v>
+        <v>1.063477767248637</v>
       </c>
       <c r="C46" s="2">
-        <v>2.936827499999326</v>
+        <v>2.879545716372734</v>
       </c>
       <c r="D46" s="2">
-        <v>1.438288705332913</v>
+        <v>1.476056745991659</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="7">
-        <v>45929</v>
+        <v>45930</v>
       </c>
       <c r="B47" s="2">
-        <v>1.062206397486472</v>
+        <v>1.092502038643798</v>
       </c>
       <c r="C47" s="2">
-        <v>2.892447244611333</v>
+        <v>2.957459797341439</v>
       </c>
       <c r="D47" s="2">
-        <v>1.475936868680455</v>
+        <v>1.508313006715899</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="7">
-        <v>45930</v>
+        <v>45931</v>
       </c>
       <c r="B48" s="2">
-        <v>1.091201265380513</v>
+        <v>1.106708129621399</v>
       </c>
       <c r="C48" s="2">
-        <v>2.970675134816483</v>
+        <v>3.041579284136568</v>
       </c>
       <c r="D48" s="2">
-        <v>1.508192668126235</v>
+        <v>1.542125431043346</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="7">
-        <v>45931</v>
+        <v>45932</v>
       </c>
       <c r="B49" s="2">
-        <v>1.10543384828651</v>
+        <v>1.137593382910526</v>
       </c>
       <c r="C49" s="2">
-        <v>3.054312784962645</v>
+        <v>3.071464028188981</v>
       </c>
       <c r="D49" s="2">
-        <v>1.542003647842151</v>
+        <v>1.586232588995289</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="7">
-        <v>45932</v>
+        <v>45933</v>
       </c>
       <c r="B50" s="2">
-        <v>1.136287060599294</v>
+        <v>1.149954305750272</v>
       </c>
       <c r="C50" s="2">
-        <v>3.083673918086981</v>
+        <v>3.156121881993007</v>
       </c>
       <c r="D50" s="2">
-        <v>1.586107284427047</v>
+        <v>1.626757235857618</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="7">
-        <v>45933</v>
+        <v>45936</v>
       </c>
       <c r="B51" s="2">
-        <v>1.148682389459768</v>
+        <v>1.180024326165145</v>
       </c>
       <c r="C51" s="2">
-        <v>3.168587492581788</v>
+        <v>3.137191306549433</v>
       </c>
       <c r="D51" s="2">
-        <v>1.626629293157687</v>
+        <v>1.672962405293818</v>
       </c>
     </row>
   </sheetData>

</xml_diff>